<commit_message>
Rename oligos to 16S-A1..A6 (6 amplicons); regenerate Excel and pages; add name map
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ao75Yp9yo6KZf9ARd9UmQz
</commit_message>
<xml_diff>
--- a/docs/primer_design/primer_order_12_16_24.xlsx
+++ b/docs/primer_design/primer_order_12_16_24.xlsx
@@ -12,7 +12,8 @@
     <sheet name="12 条池" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="16 条池" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="24 条池" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="池比较" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="名称对照" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="池比较" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -540,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -592,79 +593,86 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr"/>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>名称对照：订购名称与分析里旧名的对照。</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>颜色约定</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>蓝色字 = 输入（可以修改）：合成规模、纯化方式、母液浓度、10× 混合液体积、各引物位点内比例。黑色 = 公式，自动计算。黄色底 = 订购前需要你确认的设置。</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr"/>
-    </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>订购注意</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>1. 序列用 IUPAC 简并码（R=A/G，Y=C/T，W=A/T，M=A/C，K=G/T，S=G/C，D=A/G/T，B=C/G/T，V=A/C/G），按“混合碱基”合成，每条订一个管，不要拆成单个展开序列。订购前请确认合成商支持这些简并碱基。</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2. 序列只含基因特异部分，没有接头、UDP 或修饰；如果建库要在引物上加接头，请自己加，并重新检查 Tm 和二聚体（我没有评估带接头的版本）。</t>
+          <t>1. 序列用 IUPAC 简并码（R=A/G，Y=C/T，W=A/T，M=A/C，K=G/T，S=G/C，D=A/G/T，B=C/G/T，V=A/C/G），按“混合碱基”合成，每条订一个管，不要拆成单个展开序列。订购前请确认合成商支持这些简并碱基。</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>3. 合成规模和纯化方式不是我推荐的结果，是占位的默认值（25 nmol、标准脱盐），请按你的合成商和用量改成实际要求；含有较多简并碱基的引物，合成商可能建议更高的规模。</t>
+          <t>2. 序列只含基因特异部分，没有接头、UDP 或修饰；如果建库要在引物上加接头，请自己加，并重新检查 Tm 和二聚体（我没有评估带接头的版本）。</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>4. “订购名称”用 ASCII 字符（S5- 开头，末尾 s = 支原体补充），可以直接用于订购；“中文名”只是对应页面里的名称。</t>
+          <t>3. 合成规模和纯化方式不是我推荐的结果，是占位的默认值（25 nmol、标准脱盐），请按你的合成商和用量改成实际要求；含有较多简并碱基的引物，合成商可能建议更高的规模。</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>5. 配池：每个引物位点（共 11 个）总量相同；同位点内多条时按各自覆盖比例分，补充引物占 10%；24 条池里同位点的冗余引物（A1-F 与 V1_f；V5-R.1、V5-R.2 与 907R）按覆盖比例平分。</t>
+          <t>4. 订购名称按 6 个扩增子编号：16S-A1（V1·V2）、A2（V3）、A3（V4）、A4（V5）、A5（V6·V7）、A6（V8·V9），后面是 F（正向）/R（反向）和序号。V5 扩增子（A4）的正向引物与 V4 共用（16S-A3-F），所以 A4 只有反向引物。末尾 s = 支原体补充，.SNAP = 借鉴 Swift SNAP 的引物。名称全是 ASCII，可以直接用于订购；分析和早期页面里用过的旧名见“名称对照”工作表。</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>5. 配池：每个引物位点（共 11 个）总量相同；同位点内多条时按各自覆盖比例分，补充引物占 10%；24 条池里同位点的冗余引物（A1-F 与 V1_f；V5-R.1、V5-R.2 与 907R）按覆盖比例平分。</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
           <t>6. 这些设计是序列层面的计算结果（Greengenes 13_8 和 SILVA 128；匹配规则：最多 1 个错配、3′ 端 3 个碱基匹配），没有实验验证；退火温度建议先做梯度（大致 52–60 °C）。</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr"/>
-    </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>数据来源：docs/primer_design/order_list_levels.csv、order_list_levels_long.csv，评估见 primer_order_list_levels.html。</t>
         </is>
@@ -716,12 +724,12 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>订购名称（ASCII）</t>
+          <t>订购名称</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>中文名</t>
+          <t>分析里的旧名</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
@@ -826,12 +834,12 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>S5-A1-F</t>
+          <t>16S-A1-F</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>SMURF5-A1-F</t>
+          <t>A1-F</t>
         </is>
       </c>
       <c r="D2" s="7" t="inlineStr">
@@ -909,7 +917,11 @@
           <t>无</t>
         </is>
       </c>
-      <c r="V2" s="6" t="inlineStr"/>
+      <c r="V2" s="6" t="inlineStr">
+        <is>
+          <t>与 16S-A1-F.SNAP 同位点，24 条池同时含两者</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
@@ -917,12 +929,12 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>S5-A1-F.V1f</t>
+          <t>16S-A1-F.SNAP</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>SMURF5-A1-F.V1f（SNAP）</t>
+          <t>A1-F.V1f（SNAP）</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
@@ -1000,7 +1012,11 @@
           <t>无</t>
         </is>
       </c>
-      <c r="V3" s="6" t="inlineStr"/>
+      <c r="V3" s="6" t="inlineStr">
+        <is>
+          <t>借鉴 Swift SNAP 的引物，来源序列见其引物文件；使用前请自行确认授权</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
@@ -1008,12 +1024,12 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>S5-A1-R.1</t>
+          <t>16S-A1-R.1</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>SMURF5-A1-R.1</t>
+          <t>A1-R.1</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
@@ -1103,12 +1119,12 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>S5-A1-R.2</t>
+          <t>16S-A1-R.2</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>SMURF5-A1-R.2</t>
+          <t>A1-R.2</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
@@ -1194,12 +1210,12 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>S5-A1-R.3</t>
+          <t>16S-A1-R.3</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>SMURF5-A1-R.3</t>
+          <t>A1-R.3</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
@@ -1281,12 +1297,12 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>S5-A1-R.4s</t>
+          <t>16S-A1-R.4s</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>SMURF5-A1-R.4（补充）</t>
+          <t>A1-R.4（补充）</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
@@ -1368,12 +1384,12 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>S5-A2-F.1</t>
+          <t>16S-A2-F.1</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>SMURF5-A2-F.1</t>
+          <t>A2-F.1</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -1463,12 +1479,12 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>S5-A2-F.2s</t>
+          <t>16S-A2-F.2s</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>SMURF5-A2-F.2（补充）</t>
+          <t>A2-F.2（补充）</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -1550,12 +1566,12 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>S5-A2-R</t>
+          <t>16S-A2-R</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>SMURF5-A2-R</t>
+          <t>A2-R</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -1645,12 +1661,12 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>S5-A3-F.1</t>
+          <t>16S-A3-F.1</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>SMURF5-A3-F.1</t>
+          <t>A3-F.1</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -1732,7 +1748,11 @@
           <t>无</t>
         </is>
       </c>
-      <c r="V11" s="6" t="inlineStr"/>
+      <c r="V11" s="6" t="inlineStr">
+        <is>
+          <t>也是 V5 扩增子（A4）的正向引物，共用</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n">
@@ -1740,12 +1760,12 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>S5-A3-F.2</t>
+          <t>16S-A3-F.2</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>SMURF5-A3-F.2</t>
+          <t>A3-F.2</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -1827,7 +1847,11 @@
           <t>无</t>
         </is>
       </c>
-      <c r="V12" s="6" t="inlineStr"/>
+      <c r="V12" s="6" t="inlineStr">
+        <is>
+          <t>也是 V5 扩增子（A4）的正向引物，共用</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
@@ -1835,12 +1859,12 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>S5-A3-R</t>
+          <t>16S-A3-R</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>SMURF5-A3-R</t>
+          <t>A3-R</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -1930,12 +1954,12 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>S5-V5-R.1</t>
+          <t>16S-A4-R.1</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>SMURF5-V5-R.1</t>
+          <t>V5-R.1</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -1949,7 +1973,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>V5-R</t>
+          <t>A4-R</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -2017,7 +2041,11 @@
           <t>无</t>
         </is>
       </c>
-      <c r="V14" s="6" t="inlineStr"/>
+      <c r="V14" s="6" t="inlineStr">
+        <is>
+          <t>V5 扩增子的反向引物（正向引物是 A3-F）</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n">
@@ -2025,12 +2053,12 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>S5-V5-R.2</t>
+          <t>16S-A4-R.2</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>SMURF5-V5-R.2</t>
+          <t>V5-R.2</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
@@ -2044,7 +2072,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>V5-R</t>
+          <t>A4-R</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -2104,7 +2132,11 @@
           <t>无</t>
         </is>
       </c>
-      <c r="V15" s="6" t="inlineStr"/>
+      <c r="V15" s="6" t="inlineStr">
+        <is>
+          <t>V5 扩增子的反向引物（正向引物是 A3-F）</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n">
@@ -2112,12 +2144,12 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>S5-V5-R.907R</t>
+          <t>16S-A4-R.SNAP</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>SMURF5-V5-R.907R（SNAP）</t>
+          <t>V5-R.907R（SNAP）</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
@@ -2131,7 +2163,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>V5-R</t>
+          <t>A4-R</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -2191,7 +2223,11 @@
           <t>无</t>
         </is>
       </c>
-      <c r="V16" s="6" t="inlineStr"/>
+      <c r="V16" s="6" t="inlineStr">
+        <is>
+          <t>V5 扩增子的反向引物（正向引物是 A3-F）</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n">
@@ -2199,12 +2235,12 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>S5-A4-F.1</t>
+          <t>16S-A5-F.1</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>SMURF5-A4-F.1</t>
+          <t>A4-F.1</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
@@ -2218,7 +2254,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>A4-F</t>
+          <t>A5-F</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -2294,12 +2330,12 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>S5-A4-F.2</t>
+          <t>16S-A5-F.2</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>SMURF5-A4-F.2</t>
+          <t>A4-F.2</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
@@ -2313,7 +2349,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>A4-F</t>
+          <t>A5-F</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -2381,12 +2417,12 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>S5-A4-F.3s</t>
+          <t>16S-A5-F.3s</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>SMURF5-A4-F.3（补充）</t>
+          <t>A4-F.3（补充）</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
@@ -2400,7 +2436,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>A4-F</t>
+          <t>A5-F</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
@@ -2472,12 +2508,12 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>S5-A4-R.1</t>
+          <t>16S-A5-R.1</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>SMURF5-A4-R.1</t>
+          <t>A4-R.1</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
@@ -2491,7 +2527,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>A4-R</t>
+          <t>A5-R</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
@@ -2567,12 +2603,12 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>S5-A4-R.2s</t>
+          <t>16S-A5-R.2s</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>SMURF5-A4-R.2（补充）</t>
+          <t>A4-R.2（补充）</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
@@ -2586,7 +2622,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>A4-R</t>
+          <t>A5-R</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
@@ -2654,12 +2690,12 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>S5-A5-F.1</t>
+          <t>16S-A6-F.1</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>SMURF5-A5-F.1</t>
+          <t>A5-F.1</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
@@ -2673,7 +2709,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>A5-F</t>
+          <t>A6-F</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
@@ -2745,12 +2781,12 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>S5-A5-F.2</t>
+          <t>16S-A6-F.2</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>SMURF5-A5-F.2</t>
+          <t>A5-F.2</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -2764,7 +2800,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>A5-F</t>
+          <t>A6-F</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
@@ -2840,12 +2876,12 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>S5-A5-F.3s</t>
+          <t>16S-A6-F.3s</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>SMURF5-A5-F.3（补充）</t>
+          <t>A5-F.3（补充）</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
@@ -2859,7 +2895,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>A5-F</t>
+          <t>A6-F</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
@@ -2931,12 +2967,12 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>S5-A5-R</t>
+          <t>16S-A6-R</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>SMURF5-A5-R</t>
+          <t>A5-R</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
@@ -2950,7 +2986,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>A5-R</t>
+          <t>A6-R</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
@@ -3164,7 +3200,7 @@
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>订购名称（ASCII）</t>
+          <t>订购名称</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -3206,7 +3242,7 @@
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>S5-A1-F</t>
+          <t>16S-A1-F</t>
         </is>
       </c>
       <c r="B9" s="20" t="inlineStr">
@@ -3241,7 +3277,7 @@
     <row r="10">
       <c r="A10" s="19" t="inlineStr">
         <is>
-          <t>S5-A1-R.1</t>
+          <t>16S-A1-R.1</t>
         </is>
       </c>
       <c r="B10" s="20" t="inlineStr">
@@ -3276,7 +3312,7 @@
     <row r="11">
       <c r="A11" s="19" t="inlineStr">
         <is>
-          <t>S5-A2-F.1</t>
+          <t>16S-A2-F.1</t>
         </is>
       </c>
       <c r="B11" s="20" t="inlineStr">
@@ -3311,7 +3347,7 @@
     <row r="12">
       <c r="A12" s="19" t="inlineStr">
         <is>
-          <t>S5-A2-R</t>
+          <t>16S-A2-R</t>
         </is>
       </c>
       <c r="B12" s="20" t="inlineStr">
@@ -3346,7 +3382,7 @@
     <row r="13">
       <c r="A13" s="19" t="inlineStr">
         <is>
-          <t>S5-A3-F.1</t>
+          <t>16S-A3-F.1</t>
         </is>
       </c>
       <c r="B13" s="20" t="inlineStr">
@@ -3381,7 +3417,7 @@
     <row r="14">
       <c r="A14" s="19" t="inlineStr">
         <is>
-          <t>S5-A3-F.2</t>
+          <t>16S-A3-F.2</t>
         </is>
       </c>
       <c r="B14" s="20" t="inlineStr">
@@ -3416,7 +3452,7 @@
     <row r="15">
       <c r="A15" s="19" t="inlineStr">
         <is>
-          <t>S5-A3-R</t>
+          <t>16S-A3-R</t>
         </is>
       </c>
       <c r="B15" s="20" t="inlineStr">
@@ -3451,7 +3487,7 @@
     <row r="16">
       <c r="A16" s="19" t="inlineStr">
         <is>
-          <t>S5-V5-R.1</t>
+          <t>16S-A4-R.1</t>
         </is>
       </c>
       <c r="B16" s="20" t="inlineStr">
@@ -3461,7 +3497,7 @@
       </c>
       <c r="C16" s="19" t="inlineStr">
         <is>
-          <t>V5-R</t>
+          <t>A4-R</t>
         </is>
       </c>
       <c r="D16" s="19" t="n">
@@ -3486,7 +3522,7 @@
     <row r="17">
       <c r="A17" s="19" t="inlineStr">
         <is>
-          <t>S5-A4-F.1</t>
+          <t>16S-A5-F.1</t>
         </is>
       </c>
       <c r="B17" s="20" t="inlineStr">
@@ -3496,7 +3532,7 @@
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>A4-F</t>
+          <t>A5-F</t>
         </is>
       </c>
       <c r="D17" s="19" t="n">
@@ -3521,7 +3557,7 @@
     <row r="18">
       <c r="A18" s="19" t="inlineStr">
         <is>
-          <t>S5-A4-R.1</t>
+          <t>16S-A5-R.1</t>
         </is>
       </c>
       <c r="B18" s="20" t="inlineStr">
@@ -3531,7 +3567,7 @@
       </c>
       <c r="C18" s="19" t="inlineStr">
         <is>
-          <t>A4-R</t>
+          <t>A5-R</t>
         </is>
       </c>
       <c r="D18" s="19" t="n">
@@ -3556,7 +3592,7 @@
     <row r="19">
       <c r="A19" s="19" t="inlineStr">
         <is>
-          <t>S5-A5-F.2</t>
+          <t>16S-A6-F.2</t>
         </is>
       </c>
       <c r="B19" s="20" t="inlineStr">
@@ -3566,7 +3602,7 @@
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>A5-F</t>
+          <t>A6-F</t>
         </is>
       </c>
       <c r="D19" s="19" t="n">
@@ -3591,7 +3627,7 @@
     <row r="20">
       <c r="A20" s="19" t="inlineStr">
         <is>
-          <t>S5-A5-R</t>
+          <t>16S-A6-R</t>
         </is>
       </c>
       <c r="B20" s="20" t="inlineStr">
@@ -3601,7 +3637,7 @@
       </c>
       <c r="C20" s="19" t="inlineStr">
         <is>
-          <t>A5-R</t>
+          <t>A6-R</t>
         </is>
       </c>
       <c r="D20" s="19" t="n">
@@ -3761,7 +3797,7 @@
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>订购名称（ASCII）</t>
+          <t>订购名称</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -3803,7 +3839,7 @@
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>S5-A1-F.V1f</t>
+          <t>16S-A1-F.SNAP</t>
         </is>
       </c>
       <c r="B9" s="20" t="inlineStr">
@@ -3838,7 +3874,7 @@
     <row r="10">
       <c r="A10" s="19" t="inlineStr">
         <is>
-          <t>S5-A1-R.1</t>
+          <t>16S-A1-R.1</t>
         </is>
       </c>
       <c r="B10" s="20" t="inlineStr">
@@ -3873,7 +3909,7 @@
     <row r="11">
       <c r="A11" s="19" t="inlineStr">
         <is>
-          <t>S5-A1-R.2</t>
+          <t>16S-A1-R.2</t>
         </is>
       </c>
       <c r="B11" s="20" t="inlineStr">
@@ -3908,7 +3944,7 @@
     <row r="12">
       <c r="A12" s="19" t="inlineStr">
         <is>
-          <t>S5-A2-F.1</t>
+          <t>16S-A2-F.1</t>
         </is>
       </c>
       <c r="B12" s="20" t="inlineStr">
@@ -3943,7 +3979,7 @@
     <row r="13">
       <c r="A13" s="19" t="inlineStr">
         <is>
-          <t>S5-A2-R</t>
+          <t>16S-A2-R</t>
         </is>
       </c>
       <c r="B13" s="20" t="inlineStr">
@@ -3978,7 +4014,7 @@
     <row r="14">
       <c r="A14" s="19" t="inlineStr">
         <is>
-          <t>S5-A3-F.1</t>
+          <t>16S-A3-F.1</t>
         </is>
       </c>
       <c r="B14" s="20" t="inlineStr">
@@ -4013,7 +4049,7 @@
     <row r="15">
       <c r="A15" s="19" t="inlineStr">
         <is>
-          <t>S5-A3-F.2</t>
+          <t>16S-A3-F.2</t>
         </is>
       </c>
       <c r="B15" s="20" t="inlineStr">
@@ -4048,7 +4084,7 @@
     <row r="16">
       <c r="A16" s="19" t="inlineStr">
         <is>
-          <t>S5-A3-R</t>
+          <t>16S-A3-R</t>
         </is>
       </c>
       <c r="B16" s="20" t="inlineStr">
@@ -4083,7 +4119,7 @@
     <row r="17">
       <c r="A17" s="19" t="inlineStr">
         <is>
-          <t>S5-V5-R.1</t>
+          <t>16S-A4-R.1</t>
         </is>
       </c>
       <c r="B17" s="20" t="inlineStr">
@@ -4093,7 +4129,7 @@
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>V5-R</t>
+          <t>A4-R</t>
         </is>
       </c>
       <c r="D17" s="19" t="n">
@@ -4118,7 +4154,7 @@
     <row r="18">
       <c r="A18" s="19" t="inlineStr">
         <is>
-          <t>S5-A4-F.1</t>
+          <t>16S-A5-F.1</t>
         </is>
       </c>
       <c r="B18" s="20" t="inlineStr">
@@ -4128,7 +4164,7 @@
       </c>
       <c r="C18" s="19" t="inlineStr">
         <is>
-          <t>A4-F</t>
+          <t>A5-F</t>
         </is>
       </c>
       <c r="D18" s="19" t="n">
@@ -4153,7 +4189,7 @@
     <row r="19">
       <c r="A19" s="19" t="inlineStr">
         <is>
-          <t>S5-A4-F.3s</t>
+          <t>16S-A5-F.3s</t>
         </is>
       </c>
       <c r="B19" s="20" t="inlineStr">
@@ -4163,7 +4199,7 @@
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>A4-F</t>
+          <t>A5-F</t>
         </is>
       </c>
       <c r="D19" s="19" t="n">
@@ -4188,7 +4224,7 @@
     <row r="20">
       <c r="A20" s="19" t="inlineStr">
         <is>
-          <t>S5-A4-R.1</t>
+          <t>16S-A5-R.1</t>
         </is>
       </c>
       <c r="B20" s="20" t="inlineStr">
@@ -4198,7 +4234,7 @@
       </c>
       <c r="C20" s="19" t="inlineStr">
         <is>
-          <t>A4-R</t>
+          <t>A5-R</t>
         </is>
       </c>
       <c r="D20" s="19" t="n">
@@ -4223,7 +4259,7 @@
     <row r="21">
       <c r="A21" s="19" t="inlineStr">
         <is>
-          <t>S5-A5-F.1</t>
+          <t>16S-A6-F.1</t>
         </is>
       </c>
       <c r="B21" s="20" t="inlineStr">
@@ -4233,7 +4269,7 @@
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>A5-F</t>
+          <t>A6-F</t>
         </is>
       </c>
       <c r="D21" s="19" t="n">
@@ -4258,7 +4294,7 @@
     <row r="22">
       <c r="A22" s="19" t="inlineStr">
         <is>
-          <t>S5-A5-F.2</t>
+          <t>16S-A6-F.2</t>
         </is>
       </c>
       <c r="B22" s="20" t="inlineStr">
@@ -4268,7 +4304,7 @@
       </c>
       <c r="C22" s="19" t="inlineStr">
         <is>
-          <t>A5-F</t>
+          <t>A6-F</t>
         </is>
       </c>
       <c r="D22" s="19" t="n">
@@ -4293,7 +4329,7 @@
     <row r="23">
       <c r="A23" s="19" t="inlineStr">
         <is>
-          <t>S5-A5-F.3s</t>
+          <t>16S-A6-F.3s</t>
         </is>
       </c>
       <c r="B23" s="20" t="inlineStr">
@@ -4303,7 +4339,7 @@
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>A5-F</t>
+          <t>A6-F</t>
         </is>
       </c>
       <c r="D23" s="19" t="n">
@@ -4328,7 +4364,7 @@
     <row r="24">
       <c r="A24" s="19" t="inlineStr">
         <is>
-          <t>S5-A5-R</t>
+          <t>16S-A6-R</t>
         </is>
       </c>
       <c r="B24" s="20" t="inlineStr">
@@ -4338,7 +4374,7 @@
       </c>
       <c r="C24" s="19" t="inlineStr">
         <is>
-          <t>A5-R</t>
+          <t>A6-R</t>
         </is>
       </c>
       <c r="D24" s="19" t="n">
@@ -4498,7 +4534,7 @@
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>订购名称（ASCII）</t>
+          <t>订购名称</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -4540,7 +4576,7 @@
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>S5-A1-F</t>
+          <t>16S-A1-F</t>
         </is>
       </c>
       <c r="B9" s="20" t="inlineStr">
@@ -4575,7 +4611,7 @@
     <row r="10">
       <c r="A10" s="19" t="inlineStr">
         <is>
-          <t>S5-A1-F.V1f</t>
+          <t>16S-A1-F.SNAP</t>
         </is>
       </c>
       <c r="B10" s="20" t="inlineStr">
@@ -4610,7 +4646,7 @@
     <row r="11">
       <c r="A11" s="19" t="inlineStr">
         <is>
-          <t>S5-A1-R.1</t>
+          <t>16S-A1-R.1</t>
         </is>
       </c>
       <c r="B11" s="20" t="inlineStr">
@@ -4645,7 +4681,7 @@
     <row r="12">
       <c r="A12" s="19" t="inlineStr">
         <is>
-          <t>S5-A1-R.2</t>
+          <t>16S-A1-R.2</t>
         </is>
       </c>
       <c r="B12" s="20" t="inlineStr">
@@ -4680,7 +4716,7 @@
     <row r="13">
       <c r="A13" s="19" t="inlineStr">
         <is>
-          <t>S5-A1-R.3</t>
+          <t>16S-A1-R.3</t>
         </is>
       </c>
       <c r="B13" s="20" t="inlineStr">
@@ -4715,7 +4751,7 @@
     <row r="14">
       <c r="A14" s="19" t="inlineStr">
         <is>
-          <t>S5-A1-R.4s</t>
+          <t>16S-A1-R.4s</t>
         </is>
       </c>
       <c r="B14" s="20" t="inlineStr">
@@ -4750,7 +4786,7 @@
     <row r="15">
       <c r="A15" s="19" t="inlineStr">
         <is>
-          <t>S5-A2-F.1</t>
+          <t>16S-A2-F.1</t>
         </is>
       </c>
       <c r="B15" s="20" t="inlineStr">
@@ -4785,7 +4821,7 @@
     <row r="16">
       <c r="A16" s="19" t="inlineStr">
         <is>
-          <t>S5-A2-F.2s</t>
+          <t>16S-A2-F.2s</t>
         </is>
       </c>
       <c r="B16" s="20" t="inlineStr">
@@ -4820,7 +4856,7 @@
     <row r="17">
       <c r="A17" s="19" t="inlineStr">
         <is>
-          <t>S5-A2-R</t>
+          <t>16S-A2-R</t>
         </is>
       </c>
       <c r="B17" s="20" t="inlineStr">
@@ -4855,7 +4891,7 @@
     <row r="18">
       <c r="A18" s="19" t="inlineStr">
         <is>
-          <t>S5-A3-F.1</t>
+          <t>16S-A3-F.1</t>
         </is>
       </c>
       <c r="B18" s="20" t="inlineStr">
@@ -4890,7 +4926,7 @@
     <row r="19">
       <c r="A19" s="19" t="inlineStr">
         <is>
-          <t>S5-A3-F.2</t>
+          <t>16S-A3-F.2</t>
         </is>
       </c>
       <c r="B19" s="20" t="inlineStr">
@@ -4925,7 +4961,7 @@
     <row r="20">
       <c r="A20" s="19" t="inlineStr">
         <is>
-          <t>S5-A3-R</t>
+          <t>16S-A3-R</t>
         </is>
       </c>
       <c r="B20" s="20" t="inlineStr">
@@ -4960,7 +4996,7 @@
     <row r="21">
       <c r="A21" s="19" t="inlineStr">
         <is>
-          <t>S5-V5-R.1</t>
+          <t>16S-A4-R.1</t>
         </is>
       </c>
       <c r="B21" s="20" t="inlineStr">
@@ -4970,7 +5006,7 @@
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>V5-R</t>
+          <t>A4-R</t>
         </is>
       </c>
       <c r="D21" s="19" t="n">
@@ -4995,7 +5031,7 @@
     <row r="22">
       <c r="A22" s="19" t="inlineStr">
         <is>
-          <t>S5-V5-R.2</t>
+          <t>16S-A4-R.2</t>
         </is>
       </c>
       <c r="B22" s="20" t="inlineStr">
@@ -5005,7 +5041,7 @@
       </c>
       <c r="C22" s="19" t="inlineStr">
         <is>
-          <t>V5-R</t>
+          <t>A4-R</t>
         </is>
       </c>
       <c r="D22" s="19" t="n">
@@ -5030,7 +5066,7 @@
     <row r="23">
       <c r="A23" s="19" t="inlineStr">
         <is>
-          <t>S5-V5-R.907R</t>
+          <t>16S-A4-R.SNAP</t>
         </is>
       </c>
       <c r="B23" s="20" t="inlineStr">
@@ -5040,7 +5076,7 @@
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>V5-R</t>
+          <t>A4-R</t>
         </is>
       </c>
       <c r="D23" s="19" t="n">
@@ -5065,7 +5101,7 @@
     <row r="24">
       <c r="A24" s="19" t="inlineStr">
         <is>
-          <t>S5-A4-F.1</t>
+          <t>16S-A5-F.1</t>
         </is>
       </c>
       <c r="B24" s="20" t="inlineStr">
@@ -5075,7 +5111,7 @@
       </c>
       <c r="C24" s="19" t="inlineStr">
         <is>
-          <t>A4-F</t>
+          <t>A5-F</t>
         </is>
       </c>
       <c r="D24" s="19" t="n">
@@ -5100,7 +5136,7 @@
     <row r="25">
       <c r="A25" s="19" t="inlineStr">
         <is>
-          <t>S5-A4-F.2</t>
+          <t>16S-A5-F.2</t>
         </is>
       </c>
       <c r="B25" s="20" t="inlineStr">
@@ -5110,7 +5146,7 @@
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>A4-F</t>
+          <t>A5-F</t>
         </is>
       </c>
       <c r="D25" s="19" t="n">
@@ -5135,7 +5171,7 @@
     <row r="26">
       <c r="A26" s="19" t="inlineStr">
         <is>
-          <t>S5-A4-F.3s</t>
+          <t>16S-A5-F.3s</t>
         </is>
       </c>
       <c r="B26" s="20" t="inlineStr">
@@ -5145,7 +5181,7 @@
       </c>
       <c r="C26" s="19" t="inlineStr">
         <is>
-          <t>A4-F</t>
+          <t>A5-F</t>
         </is>
       </c>
       <c r="D26" s="19" t="n">
@@ -5170,7 +5206,7 @@
     <row r="27">
       <c r="A27" s="19" t="inlineStr">
         <is>
-          <t>S5-A4-R.1</t>
+          <t>16S-A5-R.1</t>
         </is>
       </c>
       <c r="B27" s="20" t="inlineStr">
@@ -5180,7 +5216,7 @@
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>A4-R</t>
+          <t>A5-R</t>
         </is>
       </c>
       <c r="D27" s="19" t="n">
@@ -5205,7 +5241,7 @@
     <row r="28">
       <c r="A28" s="19" t="inlineStr">
         <is>
-          <t>S5-A4-R.2s</t>
+          <t>16S-A5-R.2s</t>
         </is>
       </c>
       <c r="B28" s="20" t="inlineStr">
@@ -5215,7 +5251,7 @@
       </c>
       <c r="C28" s="19" t="inlineStr">
         <is>
-          <t>A4-R</t>
+          <t>A5-R</t>
         </is>
       </c>
       <c r="D28" s="19" t="n">
@@ -5240,7 +5276,7 @@
     <row r="29">
       <c r="A29" s="19" t="inlineStr">
         <is>
-          <t>S5-A5-F.1</t>
+          <t>16S-A6-F.1</t>
         </is>
       </c>
       <c r="B29" s="20" t="inlineStr">
@@ -5250,7 +5286,7 @@
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>A5-F</t>
+          <t>A6-F</t>
         </is>
       </c>
       <c r="D29" s="19" t="n">
@@ -5275,7 +5311,7 @@
     <row r="30">
       <c r="A30" s="19" t="inlineStr">
         <is>
-          <t>S5-A5-F.2</t>
+          <t>16S-A6-F.2</t>
         </is>
       </c>
       <c r="B30" s="20" t="inlineStr">
@@ -5285,7 +5321,7 @@
       </c>
       <c r="C30" s="19" t="inlineStr">
         <is>
-          <t>A5-F</t>
+          <t>A6-F</t>
         </is>
       </c>
       <c r="D30" s="19" t="n">
@@ -5310,7 +5346,7 @@
     <row r="31">
       <c r="A31" s="19" t="inlineStr">
         <is>
-          <t>S5-A5-F.3s</t>
+          <t>16S-A6-F.3s</t>
         </is>
       </c>
       <c r="B31" s="20" t="inlineStr">
@@ -5320,7 +5356,7 @@
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>A5-F</t>
+          <t>A6-F</t>
         </is>
       </c>
       <c r="D31" s="19" t="n">
@@ -5345,7 +5381,7 @@
     <row r="32">
       <c r="A32" s="19" t="inlineStr">
         <is>
-          <t>S5-A5-R</t>
+          <t>16S-A6-R</t>
         </is>
       </c>
       <c r="B32" s="20" t="inlineStr">
@@ -5355,7 +5391,7 @@
       </c>
       <c r="C32" s="19" t="inlineStr">
         <is>
-          <t>A5-R</t>
+          <t>A6-R</t>
         </is>
       </c>
       <c r="D32" s="19" t="n">
@@ -5436,6 +5472,634 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>订购名称</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>分析里的旧名（早期页面和文件）</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>订购名称对应的位点</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>区域</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>16S-A1-F</t>
+        </is>
+      </c>
+      <c r="B2" s="19" t="inlineStr">
+        <is>
+          <t>A1-F</t>
+        </is>
+      </c>
+      <c r="C2" s="19" t="inlineStr">
+        <is>
+          <t>A1-F</t>
+        </is>
+      </c>
+      <c r="D2" s="19" t="inlineStr">
+        <is>
+          <t>V1·V2</t>
+        </is>
+      </c>
+      <c r="E2" s="19" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="19" t="inlineStr">
+        <is>
+          <t>16S-A1-F.SNAP</t>
+        </is>
+      </c>
+      <c r="B3" s="19" t="inlineStr">
+        <is>
+          <t>A1-F.V1f（SNAP）</t>
+        </is>
+      </c>
+      <c r="C3" s="19" t="inlineStr">
+        <is>
+          <t>A1-F</t>
+        </is>
+      </c>
+      <c r="D3" s="19" t="inlineStr">
+        <is>
+          <t>V1·V2</t>
+        </is>
+      </c>
+      <c r="E3" s="19" t="inlineStr">
+        <is>
+          <t>借鉴 Swift SNAP</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="19" t="inlineStr">
+        <is>
+          <t>16S-A1-R.1</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="inlineStr">
+        <is>
+          <t>A1-R.1</t>
+        </is>
+      </c>
+      <c r="C4" s="19" t="inlineStr">
+        <is>
+          <t>A1-R</t>
+        </is>
+      </c>
+      <c r="D4" s="19" t="inlineStr">
+        <is>
+          <t>V1·V2</t>
+        </is>
+      </c>
+      <c r="E4" s="19" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>16S-A1-R.2</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>A1-R.2</t>
+        </is>
+      </c>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>A1-R</t>
+        </is>
+      </c>
+      <c r="D5" s="19" t="inlineStr">
+        <is>
+          <t>V1·V2</t>
+        </is>
+      </c>
+      <c r="E5" s="19" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>16S-A1-R.3</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>A1-R.3</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>A1-R</t>
+        </is>
+      </c>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>V1·V2</t>
+        </is>
+      </c>
+      <c r="E6" s="19" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>16S-A1-R.4s</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>A1-R.4（补充）</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>A1-R</t>
+        </is>
+      </c>
+      <c r="D7" s="19" t="inlineStr">
+        <is>
+          <t>V1·V2</t>
+        </is>
+      </c>
+      <c r="E7" s="19" t="inlineStr">
+        <is>
+          <t>支原体补充</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>16S-A2-F.1</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>A2-F.1</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="inlineStr">
+        <is>
+          <t>A2-F</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>V3</t>
+        </is>
+      </c>
+      <c r="E8" s="19" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>16S-A2-F.2s</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>A2-F.2（补充）</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>A2-F</t>
+        </is>
+      </c>
+      <c r="D9" s="19" t="inlineStr">
+        <is>
+          <t>V3</t>
+        </is>
+      </c>
+      <c r="E9" s="19" t="inlineStr">
+        <is>
+          <t>支原体补充</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>16S-A2-R</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>A2-R</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="inlineStr">
+        <is>
+          <t>A2-R</t>
+        </is>
+      </c>
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t>V3</t>
+        </is>
+      </c>
+      <c r="E10" s="19" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>16S-A3-F.1</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>A3-F.1</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="inlineStr">
+        <is>
+          <t>A3-F</t>
+        </is>
+      </c>
+      <c r="D11" s="19" t="inlineStr">
+        <is>
+          <t>V4</t>
+        </is>
+      </c>
+      <c r="E11" s="19" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>16S-A3-F.2</t>
+        </is>
+      </c>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>A3-F.2</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="inlineStr">
+        <is>
+          <t>A3-F</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>V4</t>
+        </is>
+      </c>
+      <c r="E12" s="19" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>16S-A3-R</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>A3-R</t>
+        </is>
+      </c>
+      <c r="C13" s="19" t="inlineStr">
+        <is>
+          <t>A3-R</t>
+        </is>
+      </c>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>V4</t>
+        </is>
+      </c>
+      <c r="E13" s="19" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>16S-A4-R.1</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>V5-R.1</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>A4-R</t>
+        </is>
+      </c>
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>V5</t>
+        </is>
+      </c>
+      <c r="E14" s="19" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>16S-A4-R.2</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>V5-R.2</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="inlineStr">
+        <is>
+          <t>A4-R</t>
+        </is>
+      </c>
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>V5</t>
+        </is>
+      </c>
+      <c r="E15" s="19" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="19" t="inlineStr">
+        <is>
+          <t>16S-A4-R.SNAP</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>V5-R.907R（SNAP）</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="inlineStr">
+        <is>
+          <t>A4-R</t>
+        </is>
+      </c>
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>V5</t>
+        </is>
+      </c>
+      <c r="E16" s="19" t="inlineStr">
+        <is>
+          <t>借鉴 Swift SNAP</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t>16S-A5-F.1</t>
+        </is>
+      </c>
+      <c r="B17" s="19" t="inlineStr">
+        <is>
+          <t>A4-F.1</t>
+        </is>
+      </c>
+      <c r="C17" s="19" t="inlineStr">
+        <is>
+          <t>A5-F</t>
+        </is>
+      </c>
+      <c r="D17" s="19" t="inlineStr">
+        <is>
+          <t>V6·V7</t>
+        </is>
+      </c>
+      <c r="E17" s="19" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>16S-A5-F.2</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="inlineStr">
+        <is>
+          <t>A4-F.2</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="inlineStr">
+        <is>
+          <t>A5-F</t>
+        </is>
+      </c>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>V6·V7</t>
+        </is>
+      </c>
+      <c r="E18" s="19" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>16S-A5-F.3s</t>
+        </is>
+      </c>
+      <c r="B19" s="19" t="inlineStr">
+        <is>
+          <t>A4-F.3（补充）</t>
+        </is>
+      </c>
+      <c r="C19" s="19" t="inlineStr">
+        <is>
+          <t>A5-F</t>
+        </is>
+      </c>
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t>V6·V7</t>
+        </is>
+      </c>
+      <c r="E19" s="19" t="inlineStr">
+        <is>
+          <t>支原体补充</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <t>16S-A5-R.1</t>
+        </is>
+      </c>
+      <c r="B20" s="19" t="inlineStr">
+        <is>
+          <t>A4-R.1</t>
+        </is>
+      </c>
+      <c r="C20" s="19" t="inlineStr">
+        <is>
+          <t>A5-R</t>
+        </is>
+      </c>
+      <c r="D20" s="19" t="inlineStr">
+        <is>
+          <t>V6·V7</t>
+        </is>
+      </c>
+      <c r="E20" s="19" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="19" t="inlineStr">
+        <is>
+          <t>16S-A5-R.2s</t>
+        </is>
+      </c>
+      <c r="B21" s="19" t="inlineStr">
+        <is>
+          <t>A4-R.2（补充）</t>
+        </is>
+      </c>
+      <c r="C21" s="19" t="inlineStr">
+        <is>
+          <t>A5-R</t>
+        </is>
+      </c>
+      <c r="D21" s="19" t="inlineStr">
+        <is>
+          <t>V6·V7</t>
+        </is>
+      </c>
+      <c r="E21" s="19" t="inlineStr">
+        <is>
+          <t>支原体补充</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="19" t="inlineStr">
+        <is>
+          <t>16S-A6-F.1</t>
+        </is>
+      </c>
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t>A5-F.1</t>
+        </is>
+      </c>
+      <c r="C22" s="19" t="inlineStr">
+        <is>
+          <t>A6-F</t>
+        </is>
+      </c>
+      <c r="D22" s="19" t="inlineStr">
+        <is>
+          <t>V8·V9</t>
+        </is>
+      </c>
+      <c r="E22" s="19" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>16S-A6-F.2</t>
+        </is>
+      </c>
+      <c r="B23" s="19" t="inlineStr">
+        <is>
+          <t>A5-F.2</t>
+        </is>
+      </c>
+      <c r="C23" s="19" t="inlineStr">
+        <is>
+          <t>A6-F</t>
+        </is>
+      </c>
+      <c r="D23" s="19" t="inlineStr">
+        <is>
+          <t>V8·V9</t>
+        </is>
+      </c>
+      <c r="E23" s="19" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>16S-A6-F.3s</t>
+        </is>
+      </c>
+      <c r="B24" s="19" t="inlineStr">
+        <is>
+          <t>A5-F.3（补充）</t>
+        </is>
+      </c>
+      <c r="C24" s="19" t="inlineStr">
+        <is>
+          <t>A6-F</t>
+        </is>
+      </c>
+      <c r="D24" s="19" t="inlineStr">
+        <is>
+          <t>V8·V9</t>
+        </is>
+      </c>
+      <c r="E24" s="19" t="inlineStr">
+        <is>
+          <t>支原体补充</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="19" t="inlineStr">
+        <is>
+          <t>16S-A6-R</t>
+        </is>
+      </c>
+      <c r="B25" s="19" t="inlineStr">
+        <is>
+          <t>A5-R</t>
+        </is>
+      </c>
+      <c r="C25" s="19" t="inlineStr">
+        <is>
+          <t>A6-R</t>
+        </is>
+      </c>
+      <c r="D25" s="19" t="inlineStr">
+        <is>
+          <t>V8·V9</t>
+        </is>
+      </c>
+      <c r="E25" s="19" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>